<commit_message>
Corrida | SFE-ICC | 2026-03-19 12:25:19.687225
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ICC_out.xlsx
+++ b/indicadores/SFE-ICC_out.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Correlograma" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Referencias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Correlograma" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="475">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -103,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">23/02/2026</t>
+    <t xml:space="preserve">19/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1319,6 +1320,63 @@
   </si>
   <si>
     <t xml:space="preserve">2030.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referencias de las series incluidas en la hoja Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original | serie de datos brutos transformados, se importa directo desde base de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_normal | serie original con 12 forecasts obtenidos del mejor modelo ARIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_optimista | serie original con 12 forecasts, intervalo y límite optimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_pesimista | serie original con 12 forecasts, intervalo y límite pesimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_d16 | salida D16 del X13-ARIMA-SEATS con los factores estacionales de la serie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c_c17 | salida C17 del X13-ARIMA-SEATS con pesos del irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_d12 | salida D12 del X13-ARIMA-SEATS con el componente tendencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_129600 | tendencia HP de largo plazo con un lambda de 129.600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_200 | suavizado con filtro HP usando lambda de 200, sirve para determinar PG automáticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e_ajustada | serie ajustada por estacionalidad usando el mejor modelo (LOG o NIV según el caso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_filtrada | serie ajustada por estacionalidad y corregida por irregularidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final | serie f_filtrada con o sin suavizado 2x2 según el caso (es la vieja española)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final_fct_normal | a_original_fct ajustada por D16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_tcml | tasas de cambio mensual logarítmicas de la serie g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_var_interanual | variaciones interanuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_var_mensual | variaciones mensuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h_irregular | g_final/d_d12 componente irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i_dt | g_final/d_hp_129600 desvíos respecto de la tendencia</t>
   </si>
   <si>
     <t xml:space="preserve">Coeficientes de correlación de TCML del ICA-SFE y serie específica</t>
@@ -1915,7 +1973,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.416386992472729</v>
+        <v>0.416848197861036</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1973,7 +2031,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.154577519923936</v>
+        <v>0.154555650691561</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2043,7 +2101,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0538158775071161</v>
+        <v>0.0549472260961228</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2073,7 +2131,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0609519968791809</v>
+        <v>0.0573814650025969</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -22989,200 +23047,98 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>435</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>435</v>
-      </c>
-      <c r="B2" s="1"/>
+        <v>436</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3"/>
-      <c r="B3" s="1"/>
+      <c r="A3" t="s">
+        <v>437</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>436</v>
-      </c>
-      <c r="B4" s="1"/>
+        <v>438</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>437</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>0.0852112694214978</v>
+        <v>439</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>438</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>0.105340616005332</v>
+        <v>440</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>439</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>0.140578753925489</v>
+        <v>441</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>440</v>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>0.16703677401435</v>
+        <v>442</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>441</v>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>0.216735228606375</v>
+        <v>443</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>442</v>
-      </c>
-      <c r="B10" s="1" t="n">
-        <v>0.283565832000267</v>
+        <v>444</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>443</v>
-      </c>
-      <c r="B11" s="1" t="n">
-        <v>0.347918633201051</v>
+        <v>445</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>444</v>
-      </c>
-      <c r="B12" s="1" t="n">
-        <v>0.396199609910382</v>
+        <v>446</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>445</v>
-      </c>
-      <c r="B13" s="1" t="n">
-        <v>0.416386992472729</v>
+        <v>447</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>446</v>
-      </c>
-      <c r="B14" s="1" t="n">
-        <v>0.393163477352534</v>
+        <v>448</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>447</v>
-      </c>
-      <c r="B15" s="1" t="n">
-        <v>0.310853902128841</v>
+        <v>449</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>448</v>
-      </c>
-      <c r="B16" s="1" t="n">
-        <v>0.205333541559383</v>
+        <v>450</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>449</v>
-      </c>
-      <c r="B17" s="1" t="n">
-        <v>0.103687645514777</v>
+        <v>451</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>450</v>
-      </c>
-      <c r="B18" s="1" t="n">
-        <v>0.0287367225678865</v>
+        <v>452</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>451</v>
-      </c>
-      <c r="B19" s="1" t="n">
-        <v>-0.0167149177977297</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>452</v>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>-0.05197770345364</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
         <v>453</v>
       </c>
-      <c r="B21" s="1" t="n">
-        <v>-0.0893230267131382</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>454</v>
-      </c>
-      <c r="B22" s="1" t="n">
-        <v>-0.138327231712471</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>455</v>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>-0.197033211677903</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="1"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="1"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="1"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="1"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="1"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="1"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23190,235 +23146,210 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DC0029A6-AA60-4C79-82D7-9D48C7C7FD8C}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9CEB0E64-87B9-483B-BC6E-AC617B07DB1C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B17A2A30-3E3A-49ED-91A4-D9F2C42776EE}"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>454</v>
+      </c>
+      <c r="B2" s="1"/>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+      <c r="B3" s="1"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>455</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>0.0855064173072769</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>457</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>0.106000544912307</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>458</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>0.141325861407896</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>459</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>0.167351851238328</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>460</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>0.217404866685617</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>461</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>0.284862828559486</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>462</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>0.348622745977211</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>463</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>0.396559654221316</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>464</v>
+      </c>
+      <c r="B13" s="1" t="n">
+        <v>0.416848197861036</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>465</v>
+      </c>
+      <c r="B14" s="1" t="n">
+        <v>0.393135664486906</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>466</v>
+      </c>
+      <c r="B15" s="1" t="n">
+        <v>0.310788532824196</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>467</v>
+      </c>
+      <c r="B16" s="1" t="n">
+        <v>0.20474710847241</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>468</v>
+      </c>
+      <c r="B17" s="1" t="n">
+        <v>0.103127242195577</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>469</v>
+      </c>
+      <c r="B18" s="1" t="n">
+        <v>0.0281490189768916</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>470</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>-0.0167275406820182</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>471</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>-0.0521784080780783</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>472</v>
+      </c>
+      <c r="B21" s="1" t="n">
+        <v>-0.0916439322454532</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>473</v>
+      </c>
+      <c r="B22" s="1" t="n">
+        <v>-0.140962335573203</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>474</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>-0.199581013796565</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="1"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="1"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="1"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="1"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="1"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ICC | 2026-03-20 10:33:07.020929
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ICC_out.xlsx
+++ b/indicadores/SFE-ICC_out.xlsx
@@ -110,7 +110,7 @@
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">focampo</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -23388,4 +23388,237 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
+    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
+    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D837F954-6B7E-4A89-AA1E-8EEBCDAB4C7A}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AE723BB6-EB7D-48DD-B5A9-F5C8F1BC830B}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6B0F9DA-94D4-439D-AE3E-0B0580166825}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-ICC | 2026-06-17 11:25:21.77158
</commit_message>
<xml_diff>
--- a/indicadores/SFE-ICC_out.xlsx
+++ b/indicadores/SFE-ICC_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="477">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Índice de Confianza del Consumidor (ICC) del interior</t>
+    <t xml:space="preserve">Índice de Confianza del Consumidor (ICC)</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interior del país</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,7 +110,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">21/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -1941,9 +1947,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1954,7 +1964,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1968,12 +1978,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.410618819208574</v>
+        <v>0.408002577517039</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1984,7 +1994,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2012,7 +2022,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2026,12 +2036,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.152832737496778</v>
+        <v>0.149715961763513</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2054,7 +2064,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2068,7 +2078,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2082,7 +2092,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2096,12 +2106,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0558708966948122</v>
+        <v>0.0479563281200887</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2112,7 +2122,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2126,12 +2136,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0946652726867157</v>
+        <v>0.101957673014744</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2274,10 +2284,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2290,10 +2300,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2317,66 +2327,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>35.2849464566929</v>
@@ -2429,7 +2439,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>40.3448277559055</v>
@@ -2486,7 +2496,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>38.2898687664042</v>
@@ -2543,7 +2553,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>35.3626821356633</v>
@@ -2600,7 +2610,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>40.5169213119883</v>
@@ -2657,7 +2667,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>38.5530909422746</v>
@@ -2714,7 +2724,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>40.1887549212599</v>
@@ -2771,7 +2781,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>38.7589514610092</v>
@@ -2828,7 +2838,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>42.3626265466817</v>
@@ -2885,7 +2895,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>41.4033749051718</v>
@@ -2942,7 +2952,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>48.5014421572717</v>
@@ -2999,7 +3009,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>49.0588943569554</v>
@@ -3056,7 +3066,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>45.9634498031496</v>
@@ -3115,7 +3125,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>46.4600921677009</v>
@@ -3174,7 +3184,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>42.5841111748449</v>
@@ -3233,7 +3243,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>42.8556430446194</v>
@@ -3292,7 +3302,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>41.5673982939633</v>
@@ -3351,7 +3361,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>42.4663294268449</v>
@@ -3410,7 +3420,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>38.3700656603971</v>
@@ -3469,7 +3479,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>39.3303543307087</v>
@@ -3528,7 +3538,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>38.0589570199074</v>
@@ -3587,7 +3597,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>36.6071166976221</v>
@@ -3646,7 +3656,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>32.3629289231823</v>
@@ -3705,7 +3715,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>35.6626427165354</v>
@@ -3764,7 +3774,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>42.0356167979003</v>
@@ -3823,7 +3833,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>43.6688638352024</v>
@@ -3882,7 +3892,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>39.25</v>
@@ -3941,7 +3951,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>43.33</v>
@@ -4000,7 +4010,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>40.54</v>
@@ -4059,7 +4069,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>37.88</v>
@@ -4118,7 +4128,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>38.33</v>
@@ -4177,7 +4187,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>35.46</v>
@@ -4236,7 +4246,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>33.96</v>
@@ -4295,7 +4305,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>33.66</v>
@@ -4354,7 +4364,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>33.5</v>
@@ -4413,7 +4423,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>32.79</v>
@@ -4472,7 +4482,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>30.25</v>
@@ -4531,7 +4541,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>31.67</v>
@@ -4590,7 +4600,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>33.04</v>
@@ -4649,7 +4659,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>28.54</v>
@@ -4708,7 +4718,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>29.96</v>
@@ -4767,7 +4777,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>28.15</v>
@@ -4826,7 +4836,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>32.13</v>
@@ -4885,7 +4895,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>34</v>
@@ -4944,7 +4954,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>31.08</v>
@@ -5003,7 +5013,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>35.33</v>
@@ -5062,7 +5072,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>38.83</v>
@@ -5121,7 +5131,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>37.58</v>
@@ -5180,7 +5190,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>40.63</v>
@@ -5239,7 +5249,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>39.17</v>
@@ -5298,7 +5308,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>38.76</v>
@@ -5357,7 +5367,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>38.56</v>
@@ -5416,7 +5426,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>43.63</v>
@@ -5475,7 +5485,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>55.14</v>
@@ -5534,7 +5544,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>53.65</v>
@@ -5593,7 +5603,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>55.04</v>
@@ -5652,7 +5662,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>49.92</v>
@@ -5711,7 +5721,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>49.75</v>
@@ -5770,7 +5780,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>52.22</v>
@@ -5829,7 +5839,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>50.08</v>
@@ -5888,7 +5898,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>55.4583333333333</v>
@@ -5947,7 +5957,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>59.9166666666667</v>
@@ -6006,7 +6016,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>57.5</v>
@@ -6065,7 +6075,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>49.7916666666667</v>
@@ -6124,7 +6134,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>51.875</v>
@@ -6183,7 +6193,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>48.5833333333333</v>
@@ -6242,7 +6252,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>51.2083333333333</v>
@@ -6301,7 +6311,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>48.0514096185738</v>
@@ -6360,7 +6370,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>47.5</v>
@@ -6419,7 +6429,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>52.4166666666667</v>
@@ -6478,7 +6488,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>55.9166666666667</v>
@@ -6537,7 +6547,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>51.25</v>
@@ -6596,7 +6606,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>58.2916666666667</v>
@@ -6655,7 +6665,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>56.5416666666667</v>
@@ -6714,7 +6724,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>59.625</v>
@@ -6773,7 +6783,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>51.125</v>
@@ -6832,7 +6842,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>55</v>
@@ -6891,7 +6901,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>49.75</v>
@@ -6950,7 +6960,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>49.7937293729373</v>
@@ -7009,7 +7019,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>54.25</v>
@@ -7068,7 +7078,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>51.2916666666667</v>
@@ -7127,7 +7137,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>49.0416666666667</v>
@@ -7186,7 +7196,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>53.7916666666667</v>
@@ -7245,7 +7255,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>53</v>
@@ -7304,7 +7314,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>57.013201320132</v>
@@ -7363,7 +7373,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>55.8333333333333</v>
@@ -7422,7 +7432,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>59.0833333333333</v>
@@ -7481,7 +7491,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>55.5833333333333</v>
@@ -7540,7 +7550,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>56.4166666666667</v>
@@ -7599,7 +7609,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>58.8333333333333</v>
@@ -7658,7 +7668,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>59.1666666666667</v>
@@ -7717,7 +7727,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>56.7083333333333</v>
@@ -7776,7 +7786,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>57.75</v>
@@ -7835,7 +7845,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>60.9583333333333</v>
@@ -7894,7 +7904,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>60.2083333333333</v>
@@ -7953,7 +7963,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>59.0381426202322</v>
@@ -8012,7 +8022,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>59.375</v>
@@ -8071,7 +8081,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>59.452736318408</v>
@@ -8130,7 +8140,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>58.6666666666667</v>
@@ -8189,7 +8199,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>50.75</v>
@@ -8248,7 +8258,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>54.6666666666667</v>
@@ -8307,7 +8317,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>52.1558872305141</v>
@@ -8366,7 +8376,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>51.4166666666667</v>
@@ -8425,7 +8435,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>50.0416666666667</v>
@@ -8484,7 +8494,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>50.125</v>
@@ -8543,7 +8553,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>50</v>
@@ -8602,7 +8612,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>53.2083333333333</v>
@@ -8661,7 +8671,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>50.7916666666667</v>
@@ -8720,7 +8730,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>56.2083333333333</v>
@@ -8779,7 +8789,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>50.4975124378109</v>
@@ -8838,7 +8848,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>46.369396</v>
@@ -8897,7 +8907,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>46.43367</v>
@@ -8956,7 +8966,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>40.562675</v>
@@ -9015,7 +9025,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>38.696373</v>
@@ -9074,7 +9084,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>39.4897</v>
@@ -9133,7 +9143,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>43.538647</v>
@@ -9192,7 +9202,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>42.879219</v>
@@ -9251,7 +9261,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>38.986355</v>
@@ -9310,7 +9320,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>40.086418</v>
@@ -9369,7 +9379,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>36.921795</v>
@@ -9428,7 +9438,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>42.696358</v>
@@ -9487,7 +9497,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>38.904831</v>
@@ -9546,7 +9556,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>38.600853</v>
@@ -9605,7 +9615,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>37.844254</v>
@@ -9664,7 +9674,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>39.705162</v>
@@ -9723,7 +9733,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>39.706558</v>
@@ -9782,7 +9792,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>42.166668</v>
@@ -9841,7 +9851,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>39.483002</v>
@@ -9900,7 +9910,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>42.400566</v>
@@ -9959,7 +9969,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>39.448357</v>
@@ -10018,7 +10028,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>39.616119</v>
@@ -10077,7 +10087,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>40.603619</v>
@@ -10136,7 +10146,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>44.659039</v>
@@ -10195,7 +10205,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>42.972458</v>
@@ -10254,7 +10264,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>39.820076</v>
@@ -10313,7 +10323,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>41.536827</v>
@@ -10372,7 +10382,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>44.601749</v>
@@ -10431,7 +10441,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>47.545498</v>
@@ -10490,7 +10500,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>47.811062</v>
@@ -10549,7 +10559,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>48.894032</v>
@@ -10608,7 +10618,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>49.306625</v>
@@ -10667,7 +10677,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>50.076218</v>
@@ -10726,7 +10736,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>54.650867</v>
@@ -10785,7 +10795,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>52.959503</v>
@@ -10844,7 +10854,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>54.109241</v>
@@ -10903,7 +10913,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>52.565105</v>
@@ -10962,7 +10972,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>56.432976</v>
@@ -11021,7 +11031,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>54.639572</v>
@@ -11080,7 +11090,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>55.70652</v>
@@ -11139,7 +11149,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>52.693089</v>
@@ -11198,7 +11208,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>55.709389</v>
@@ -11257,7 +11267,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>55.086208</v>
@@ -11316,7 +11326,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>56.532921</v>
@@ -11375,7 +11385,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>56.427101</v>
@@ -11434,7 +11444,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>54.449589</v>
@@ -11493,7 +11503,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>53.870884</v>
@@ -11552,7 +11562,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>56.014942</v>
@@ -11611,7 +11621,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>51.633739</v>
@@ -11670,7 +11680,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>50.264969</v>
@@ -11729,7 +11739,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>43.068535</v>
@@ -11788,7 +11798,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>45.898846</v>
@@ -11847,7 +11857,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>45.776081</v>
@@ -11906,7 +11916,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>45.064598</v>
@@ -11965,7 +11975,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>45.110085</v>
@@ -12024,7 +12034,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>39.854519</v>
@@ -12083,7 +12093,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>42.652328</v>
@@ -12142,7 +12152,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>42.2299</v>
@@ -12201,7 +12211,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>44.318775</v>
@@ -12260,7 +12270,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>47.759857</v>
@@ -12319,7 +12329,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>45.544819</v>
@@ -12378,7 +12388,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>45.814133</v>
@@ -12437,7 +12447,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>44.354424</v>
@@ -12496,7 +12506,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>42.473545</v>
@@ -12555,7 +12565,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>45.157135</v>
@@ -12614,7 +12624,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>45.641026</v>
@@ -12673,7 +12683,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>49.0755</v>
@@ -12732,7 +12742,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>48.827728</v>
@@ -12791,7 +12801,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>50.254063</v>
@@ -12850,7 +12860,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>49.742001</v>
@@ -12909,7 +12919,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>43.77898</v>
@@ -12968,7 +12978,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>43.514271</v>
@@ -13027,7 +13037,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>35.346584</v>
@@ -13086,7 +13096,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>33.695091</v>
@@ -13145,7 +13155,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>36.509773</v>
@@ -13204,7 +13214,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>36.493374</v>
@@ -13263,7 +13273,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>40.76963</v>
@@ -13322,7 +13332,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>43.954758</v>
@@ -13381,7 +13391,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>42.758087</v>
@@ -13440,7 +13450,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>40.945389</v>
@@ -13499,7 +13509,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>44.056747</v>
@@ -13558,7 +13568,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>44.508743</v>
@@ -13617,7 +13627,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>45.25463</v>
@@ -13676,7 +13686,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>49.344929</v>
@@ -13735,7 +13745,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>48.508228</v>
@@ -13794,7 +13804,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>52.739201</v>
@@ -13853,7 +13863,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>52.18</v>
@@ -13912,7 +13922,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>57.01</v>
@@ -13971,7 +13981,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>54.413292</v>
@@ -14030,7 +14040,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>55.061348</v>
@@ -14089,7 +14099,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>55.214725</v>
@@ -14148,7 +14158,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>55.240288</v>
@@ -14207,7 +14217,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>56.726284</v>
@@ -14266,7 +14276,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>61.081013</v>
@@ -14325,7 +14335,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>57.671337</v>
@@ -14384,7 +14394,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>53.533028</v>
@@ -14443,7 +14453,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>49.323635</v>
@@ -14502,7 +14512,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>51.572086</v>
@@ -14561,7 +14571,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>45.56493</v>
@@ -14620,7 +14630,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>44.732094</v>
@@ -14679,7 +14689,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>46.919731</v>
@@ -14738,7 +14748,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>49.564102</v>
@@ -14797,7 +14807,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>46.417564</v>
@@ -14856,7 +14866,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>47.853149</v>
@@ -14915,7 +14925,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>50.598022</v>
@@ -14974,7 +14984,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>46.345257</v>
@@ -15033,7 +15043,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>48.92</v>
@@ -15092,7 +15102,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>49.4306425</v>
@@ -15151,7 +15161,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>43.9931653333333</v>
@@ -15210,7 +15220,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>45.807209</v>
@@ -15269,7 +15279,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>49.17</v>
@@ -15328,7 +15338,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>49.3260748333333</v>
@@ -15387,7 +15397,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>45.597485</v>
@@ -15446,7 +15456,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>46.909668</v>
@@ -15505,7 +15515,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>50.877193</v>
@@ -15564,7 +15574,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>56.125576</v>
@@ -15623,7 +15633,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>55.989582</v>
@@ -15682,7 +15692,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>55.944962</v>
@@ -15741,7 +15751,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>47.984921</v>
@@ -15800,7 +15810,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>46.582546</v>
@@ -15859,7 +15869,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>46.729462</v>
@@ -15918,7 +15928,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>45.794872</v>
@@ -15977,7 +15987,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>41.912525</v>
@@ -16036,7 +16046,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>39.289448</v>
@@ -16095,7 +16105,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>41.640865</v>
@@ -16154,7 +16164,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>39.859596</v>
@@ -16213,7 +16223,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>39.097549</v>
@@ -16272,7 +16282,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>35.798664</v>
@@ -16331,7 +16341,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>33.397339</v>
@@ -16390,7 +16400,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>35.007851</v>
@@ -16449,7 +16459,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>37.532299</v>
@@ -16508,7 +16518,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>37.283386</v>
@@ -16567,7 +16577,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>37.906048</v>
@@ -16626,7 +16636,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>37.551125</v>
@@ -16685,7 +16695,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>35.054081</v>
@@ -16744,7 +16754,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>38.760288</v>
@@ -16803,7 +16813,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>42.030075</v>
@@ -16862,7 +16872,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>46.286369</v>
@@ -16921,7 +16931,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>41.653904</v>
@@ -16980,7 +16990,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>42.928135</v>
@@ -17039,7 +17049,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>44.928097</v>
@@ -17098,7 +17108,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>40.201324</v>
@@ -17157,7 +17167,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>43.087265</v>
@@ -17216,7 +17226,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>42.43119</v>
@@ -17275,7 +17285,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>39.283894</v>
@@ -17334,7 +17344,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>39.513252</v>
@@ -17393,7 +17403,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>38.880329</v>
@@ -17452,7 +17462,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>38.706806</v>
@@ -17511,7 +17521,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>37.996941</v>
@@ -17570,7 +17580,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>39.397434</v>
@@ -17629,7 +17639,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>41.243591</v>
@@ -17688,7 +17698,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>39.111454</v>
@@ -17747,7 +17757,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>36.406895</v>
@@ -17806,7 +17816,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>39.519032</v>
@@ -17865,7 +17875,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>38.549717</v>
@@ -17924,7 +17934,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>36.566204</v>
@@ -17983,7 +17993,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>35.647427</v>
@@ -18042,7 +18052,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>36.210472</v>
@@ -18101,7 +18111,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>32.686337</v>
@@ -18160,7 +18170,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>35.394264</v>
@@ -18219,7 +18229,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>34.36198</v>
@@ -18278,7 +18288,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>35.346153</v>
@@ -18337,7 +18347,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>39.302147</v>
@@ -18396,7 +18406,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>40.144356</v>
@@ -18455,7 +18465,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>39.166668</v>
@@ -18514,7 +18524,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>39.3652</v>
@@ -18573,7 +18583,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>37.628998</v>
@@ -18632,7 +18642,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>38.888889</v>
@@ -18691,7 +18701,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>38.11</v>
@@ -18750,7 +18760,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>36.16798</v>
@@ -18809,7 +18819,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>34.61</v>
@@ -18868,7 +18878,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>36.623932</v>
@@ -18927,7 +18937,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>37.417</v>
@@ -18986,7 +18996,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>31.653225</v>
@@ -19045,7 +19055,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>36.586987</v>
@@ -19104,7 +19114,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>36.061508</v>
@@ -19163,7 +19173,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>34.656086</v>
@@ -19222,7 +19232,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>34.266666</v>
@@ -19281,7 +19291,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>35.921223</v>
@@ -19340,7 +19350,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>38.12</v>
@@ -19399,7 +19409,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>37.06</v>
@@ -19458,7 +19468,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>37.28</v>
@@ -19517,7 +19527,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>38.585858</v>
@@ -19576,7 +19586,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>38.704426</v>
@@ -19635,7 +19645,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>40.888889</v>
@@ -19694,7 +19704,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>43.320614</v>
@@ -19753,7 +19763,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>43.41346</v>
@@ -19812,7 +19822,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>42.562378</v>
@@ -19871,7 +19881,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>44.68504</v>
@@ -19930,7 +19940,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>46.712688</v>
@@ -19989,7 +19999,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>42.236328</v>
@@ -20048,7 +20058,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>40.277779</v>
@@ -20107,7 +20117,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>43.058285</v>
@@ -20166,7 +20176,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>41.777569</v>
@@ -20225,7 +20235,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>39.47979</v>
@@ -20284,7 +20294,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>42.906067</v>
@@ -20343,7 +20353,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>44.757515</v>
@@ -20402,7 +20412,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>44.072998</v>
@@ -20461,7 +20471,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>46.830986</v>
@@ -20520,7 +20530,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>41.699474</v>
@@ -20579,7 +20589,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>48.20039</v>
@@ -20638,7 +20648,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>53.519974</v>
@@ -20697,7 +20707,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>52.008034</v>
@@ -20756,7 +20766,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>54.388561</v>
@@ -20815,7 +20825,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>52.298279</v>
@@ -20874,7 +20884,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>50.281086</v>
@@ -20933,7 +20943,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>49.524281</v>
@@ -20992,7 +21002,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>51.633987</v>
@@ -21051,7 +21061,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>50.183334</v>
@@ -21110,7 +21120,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>49.900795</v>
@@ -21169,7 +21179,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>46.374672</v>
@@ -21228,7 +21238,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>44.646366</v>
@@ -21287,7 +21297,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>47.965118</v>
@@ -21346,7 +21356,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>51.513672</v>
@@ -21405,7 +21415,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>47.485207</v>
@@ -21464,7 +21474,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>51.236355</v>
@@ -21523,7 +21533,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>50.078175</v>
@@ -21582,7 +21592,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>50.709541</v>
@@ -21641,7 +21651,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>45.3484840393066</v>
@@ -21700,7 +21710,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>45.3947372436523</v>
@@ -21759,7 +21769,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B331" s="2"/>
       <c r="C331" s="3" t="n">
@@ -21792,7 +21802,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B332" s="2"/>
       <c r="C332" s="3" t="n">
@@ -21825,7 +21835,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B333" s="2"/>
       <c r="C333" s="3" t="n">
@@ -21858,7 +21868,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B334" s="2"/>
       <c r="C334" s="3" t="n">
@@ -21891,7 +21901,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B335" s="2"/>
       <c r="C335" s="3" t="n">
@@ -21924,7 +21934,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B336" s="2"/>
       <c r="C336" s="3" t="n">
@@ -21957,7 +21967,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B337" s="2"/>
       <c r="C337" s="3" t="n">
@@ -21990,7 +22000,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B338" s="2"/>
       <c r="C338" s="3" t="n">
@@ -22023,7 +22033,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B339" s="2"/>
       <c r="C339" s="3" t="n">
@@ -22056,7 +22066,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B340" s="2"/>
       <c r="C340" s="3" t="n">
@@ -22089,7 +22099,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B341" s="2"/>
       <c r="C341" s="3" t="n">
@@ -22122,7 +22132,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B342" s="2"/>
       <c r="C342" s="3" t="n">
@@ -22155,7 +22165,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B343" s="2"/>
       <c r="C343" s="3"/>
@@ -22178,7 +22188,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B344" s="2"/>
       <c r="C344" s="3"/>
@@ -22201,7 +22211,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B345" s="2"/>
       <c r="C345" s="3"/>
@@ -22224,7 +22234,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B346" s="2"/>
       <c r="C346" s="3"/>
@@ -22247,7 +22257,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B347" s="2"/>
       <c r="C347" s="3"/>
@@ -22270,7 +22280,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B348" s="2"/>
       <c r="C348" s="3"/>
@@ -22293,7 +22303,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B349" s="2"/>
       <c r="C349" s="3"/>
@@ -22316,7 +22326,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B350" s="2"/>
       <c r="C350" s="3"/>
@@ -22339,7 +22349,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B351" s="2"/>
       <c r="C351" s="3"/>
@@ -22362,7 +22372,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B352" s="2"/>
       <c r="C352" s="3"/>
@@ -22385,7 +22395,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B353" s="2"/>
       <c r="C353" s="3"/>
@@ -22408,7 +22418,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B354" s="2"/>
       <c r="C354" s="3"/>
@@ -22431,7 +22441,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B355" s="2"/>
       <c r="C355" s="3"/>
@@ -22454,7 +22464,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B356" s="2"/>
       <c r="C356" s="3"/>
@@ -22477,7 +22487,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B357" s="2"/>
       <c r="C357" s="3"/>
@@ -22500,7 +22510,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B358" s="2"/>
       <c r="C358" s="3"/>
@@ -22523,7 +22533,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B359" s="2"/>
       <c r="C359" s="3"/>
@@ -22546,7 +22556,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B360" s="2"/>
       <c r="C360" s="3"/>
@@ -22569,7 +22579,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B361" s="2"/>
       <c r="C361" s="3"/>
@@ -22592,7 +22602,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B362" s="2"/>
       <c r="C362" s="3"/>
@@ -22615,7 +22625,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B363" s="2"/>
       <c r="C363" s="3"/>
@@ -22638,7 +22648,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B364" s="2"/>
       <c r="C364" s="3"/>
@@ -22661,7 +22671,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B365" s="2"/>
       <c r="C365" s="3"/>
@@ -22684,7 +22694,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B366" s="2"/>
       <c r="C366" s="3"/>
@@ -22707,7 +22717,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B367" s="2"/>
       <c r="C367" s="3"/>
@@ -22730,7 +22740,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B368" s="2"/>
       <c r="C368" s="3"/>
@@ -22753,7 +22763,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B369" s="2"/>
       <c r="C369" s="3"/>
@@ -22776,7 +22786,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B370" s="2"/>
       <c r="C370" s="3"/>
@@ -22799,7 +22809,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B371" s="2"/>
       <c r="C371" s="3"/>
@@ -22822,7 +22832,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B372" s="2"/>
       <c r="C372" s="3"/>
@@ -22845,7 +22855,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B373" s="2"/>
       <c r="C373" s="3"/>
@@ -22868,7 +22878,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B374" s="2"/>
       <c r="C374" s="3"/>
@@ -22891,7 +22901,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B375" s="2"/>
       <c r="C375" s="3"/>
@@ -22914,7 +22924,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B376" s="2"/>
       <c r="C376" s="3"/>
@@ -22937,7 +22947,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B377" s="2"/>
       <c r="C377" s="3"/>
@@ -22960,7 +22970,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B378" s="2"/>
       <c r="C378" s="3"/>
@@ -22983,7 +22993,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B379" s="2"/>
       <c r="C379" s="3"/>
@@ -23006,7 +23016,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B380" s="2"/>
       <c r="C380" s="3"/>
@@ -23029,7 +23039,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B381" s="2"/>
       <c r="C381" s="3"/>
@@ -23052,7 +23062,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B382" s="2"/>
       <c r="C382" s="3"/>
@@ -23075,7 +23085,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B383" s="2"/>
       <c r="C383" s="3"/>
@@ -23098,7 +23108,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B384" s="2"/>
       <c r="C384" s="3"/>
@@ -23121,7 +23131,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B385" s="2"/>
       <c r="C385" s="3"/>
@@ -23155,97 +23165,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
     </row>
   </sheetData>
@@ -23269,7 +23279,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -23279,160 +23289,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>0.0817840575608566</v>
+        <v>0.0800307020584612</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>0.105675918620745</v>
+        <v>0.103867812071445</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.148833470644739</v>
+        <v>0.146997604111266</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.178816151109018</v>
+        <v>0.177109261784395</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.22287594958254</v>
+        <v>0.221845383328977</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.285173807727125</v>
+        <v>0.286329992138964</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.350233081693354</v>
+        <v>0.353245523340726</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.395327825590375</v>
+        <v>0.396244268418412</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.410618819208574</v>
+        <v>0.408002577517039</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.390938278372403</v>
+        <v>0.386931469078844</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.31132738838613</v>
+        <v>0.309302545385105</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.202935076848266</v>
+        <v>0.202130458347628</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.103821056463526</v>
+        <v>0.103818462465247</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.0317591184794891</v>
+        <v>0.0340832852088158</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>-0.0181996467830705</v>
+        <v>-0.0140586236566624</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>-0.0585241484585947</v>
+        <v>-0.0552549091075324</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0956276808524674</v>
+        <v>-0.0937457376642791</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.142195820291896</v>
+        <v>-0.143116926040559</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.197869460483047</v>
+        <v>-0.200458127113234</v>
       </c>
     </row>
     <row r="24">

</xml_diff>